<commit_message>
added more excersises and mistakes. deleted in miluli the data validation the 3 different waves.
</commit_message>
<xml_diff>
--- a/מילולי.xlsx
+++ b/מילולי.xlsx
@@ -8,17 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dvir\psychometricInvestigationWithGit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9A35717-54C6-44E9-B5DB-78156BAEAB7C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A4A7908-D878-4915-9E07-A32EF8D30C94}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="דוגמית לטאב" sheetId="14" r:id="rId1"/>
     <sheet name="אנלוגיות" sheetId="15" r:id="rId2"/>
+    <sheet name="הבנת הנקרא" sheetId="18" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">אנלוגיות!$B$2:$G$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'דוגמית לטאב'!$B$2:$G$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'הבנת הנקרא'!$B$2:$G$2</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -30,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="49">
   <si>
     <t>למה טעיתי</t>
   </si>
@@ -90,6 +92,93 @@
   </si>
   <si>
     <t>לשים לב לקטגוריות הלשוניות של המילים ולא להיות פזיז אם יש תשובות שקרובות</t>
+  </si>
+  <si>
+    <t>הסתכלתי על שורש המילה והבנתי מה היא אמורה להביע</t>
+  </si>
+  <si>
+    <t>ספר חשיבה מילולית</t>
+  </si>
+  <si>
+    <t>עמוד 49 שאלה 3</t>
+  </si>
+  <si>
+    <t>כי לא התעמקתי מספיק בקטע ולא חשבתי על זה שמה שכתוב הוא כן באוצר מילים משובח.</t>
+  </si>
+  <si>
+    <t>הבנה</t>
+  </si>
+  <si>
+    <t>אתעמק יותר בקטע ואשים לב למילים.</t>
+  </si>
+  <si>
+    <t>עמוד 49 שאלה 4</t>
+  </si>
+  <si>
+    <t>קראתי את משפט פתיחת הפסקה במהירות ואחר כך ברפרוף</t>
+  </si>
+  <si>
+    <t>כי מיהרתי ולא חשבתי על כך שהתשובה כללית מדי.</t>
+  </si>
+  <si>
+    <t>אעשה את השאלות בתשומת לב ולא אסמן תשובות כלליות מדי.</t>
+  </si>
+  <si>
+    <t>עמוד 51 שאלה 3</t>
+  </si>
+  <si>
+    <t>קראתי את המשפט לפני והבנתי שהתשובה צריכה להיות לפני</t>
+  </si>
+  <si>
+    <t>לא חשבתי בהיגיון וסימנתי כמו רובוט.</t>
+  </si>
+  <si>
+    <t>לשים לב להיגיון שבדברים ולא רק לחשוב שמילה מתייחסת למה שהכי קרוב אליה.</t>
+  </si>
+  <si>
+    <t>עמוד 51 שאלה 5</t>
+  </si>
+  <si>
+    <t>לא קראתי את כל הטקסט ופסלתי תשובות</t>
+  </si>
+  <si>
+    <t>כי לא השתמשתי בשיטת תיאום ציפיות ולא שמתי לב  שסייבר סקאוטינג מופיע כמעט בכל הפסקאות.</t>
+  </si>
+  <si>
+    <t>לזכור להשתמש בשיטת תיאום ציפיות ולשים לב שהתשובה לשאלות נושא הוא מה שמופיע בהכי הרבה פסקאות.</t>
+  </si>
+  <si>
+    <t>קראתי את הפסקה בזריזות</t>
+  </si>
+  <si>
+    <t>עמוד 54 שאלה 1</t>
+  </si>
+  <si>
+    <t>רפרפתי יותר מדי ולא התעמקתי בפסקה מספיק.</t>
+  </si>
+  <si>
+    <t>לקרוא את הפסקה יותר בעיון.</t>
+  </si>
+  <si>
+    <t>סימנתי תשובה שהופיעה לפני מילת ההתייחסות</t>
+  </si>
+  <si>
+    <t>עמוד 55 שאלה 2</t>
+  </si>
+  <si>
+    <t>בגלל שלא הצבתי את התשובה במשפט ולא חשבתי אם התשובה מסתדרת לפי ההיגיון.</t>
+  </si>
+  <si>
+    <t>להציב במקרה שמתלבטים בין תשובות.</t>
+  </si>
+  <si>
+    <t>עמוד 55 שאלה 4</t>
+  </si>
+  <si>
+    <t>לא שמתי לב שרוב הטקסט הוא על הטלת המגבלות ולא סתם על ניצול יתר.</t>
+  </si>
+  <si>
+    <t>לשים לב ולתאם ציפיות כמו שצריך ולא ליפול בפח על נושאים שהוצגו בקצרה בקטע.</t>
   </si>
 </sst>
 </file>
@@ -475,6 +564,14 @@
   </sheetData>
   <autoFilter ref="B2:G2" xr:uid="{87CB5822-66D4-452B-A3EB-3E11EDA85BE8}"/>
   <dataConsolidate/>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4:C1048576" xr:uid="{CDD049C4-F807-47D0-91DE-F5EE07803ADA}">
+      <formula1>"ספר חשיבה פסיכומטרית, ספר חשיבה מילולית, בחנים חמים מהתנור, סימולציה 1, סימולציה 2, סימולציה 3, סימולציה 4, סימולציה 5, סימולציה 6, סימולציה 7, סימולציה 8, סימולציה 9"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4:F1048576" xr:uid="{E7E9C9DB-8833-40B5-BB80-A8DFB85B06C6}">
+      <formula1>"ידע, הבנה, כאפה"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -2234,7 +2331,7 @@
   <dataConsolidate/>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4:C1048576" xr:uid="{1044AE8F-1B9C-4E47-A357-77C52A537DE2}">
-      <formula1>"ספר חשיבה פסיכומטרית, ספר חשיבה מילולית, גל 1, גל 2, גל 3, בחנים חמים מהתנור, סימולציה 1, סימולציה 2, סימולציה 3, סימולציה 4, סימולציה 5, סימולציה 6, סימולציה 7, סימולציה 8, סימולציה 9"</formula1>
+      <formula1>"ספר חשיבה פסיכומטרית, ספר חשיבה מילולית, בחנים חמים מהתנור, סימולציה 1, סימולציה 2, סימולציה 3, סימולציה 4, סימולציה 5, סימולציה 6, סימולציה 7, סימולציה 8, סימולציה 9"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4:F1048576" xr:uid="{C68152B5-1B1C-4558-8E32-BAE65DCD124F}">
       <formula1>"ידע, הבנה, כאפה"</formula1>
@@ -2243,4 +2340,209 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD3A6F25-0A04-4919-B9CF-E9C8E699BA69}">
+  <dimension ref="B1:G10"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="40.69921875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="18.69921875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="17.69921875" style="2" customWidth="1"/>
+    <col min="5" max="5" width="40.69921875" style="2" customWidth="1"/>
+    <col min="6" max="6" width="17.69921875" style="2" customWidth="1"/>
+    <col min="7" max="7" width="40.69921875" style="2" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B1"/>
+      <c r="C1"/>
+      <c r="D1"/>
+      <c r="E1"/>
+      <c r="F1"/>
+      <c r="G1"/>
+    </row>
+    <row r="2" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B3"/>
+      <c r="C3"/>
+      <c r="D3"/>
+      <c r="E3"/>
+      <c r="F3"/>
+      <c r="G3"/>
+    </row>
+    <row r="4" spans="2:7" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="B4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="B5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="2:7" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="B6" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" ht="41.4" x14ac:dyDescent="0.25">
+      <c r="B7" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B8" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="9" spans="2:7" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="B9" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10" spans="2:7" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="B10" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="B2:G2" xr:uid="{87CB5822-66D4-452B-A3EB-3E11EDA85BE8}"/>
+  <dataConsolidate/>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4:F1048576" xr:uid="{1094EA4C-A94E-471C-8BAA-B47A39D6F3CE}">
+      <formula1>"ידע, הבנה, כאפה"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4:C1048576" xr:uid="{626D3078-87D5-4240-B6D5-787867011455}">
+      <formula1>"ספר חשיבה פסיכומטרית, ספר חשיבה מילולית, בחנים חמים מהתנור, סימולציה 1, סימולציה 2, סימולציה 3, סימולציה 4, סימולציה 5, סימולציה 6, סימולציה 7, סימולציה 8, סימולציה 9"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>